<commit_message>
lab t2 s1 aula 20/03 - recursão e Quicksort
</commit_message>
<xml_diff>
--- a/2026_1_lab_t2_s1/nosso_vetor/grafico_logaritmo.xlsx
+++ b/2026_1_lab_t2_s1/nosso_vetor/grafico_logaritmo.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andreia\Documents\workspaces\2026_1_cic203\2026_1_lab_t2_s1\nosso_vetor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{009C6A0D-F6D0-41DA-A038-F16C9D0CE2CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0196D7-58AE-47A0-BB2C-246AA34E4738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12252" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12252" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Planilha1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
   <si>
     <t>x</t>
   </si>
@@ -45,6 +46,15 @@
   </si>
   <si>
     <t>log 10 x</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>n.lgn</t>
+  </si>
+  <si>
+    <t>n.n</t>
   </si>
 </sst>
 </file>
@@ -565,7 +575,594 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Planilha1!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>n</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Planilha1!$C$2:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Planilha1!$D$2:$D$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-BBDA-4156-9AFC-ADF98A0B995C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Planilha1!$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>n.lgn</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Planilha1!$C$2:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Planilha1!$E$2:$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>33.219280948873624</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>86.438561897747249</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>147.20671786825557</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>212.8771237954945</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>282.1928094887362</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-BBDA-4156-9AFC-ADF98A0B995C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Planilha1!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>n.n</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Planilha1!$C$2:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Planilha1!$F$2:$F$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1600</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2500</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-BBDA-4156-9AFC-ADF98A0B995C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1683013343"/>
+        <c:axId val="1682997983"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1683013343"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1682997983"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1682997983"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1683013343"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1121,6 +1718,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1142,6 +2255,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D19C80C-7A7A-333C-B518-DB4434B74B02}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>583223</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>96714</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>322385</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>123091</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB3362FC-BB36-937E-9EBB-756A6F23D2C9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1521,4 +2675,114 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BD492F2-D711-4B1D-9F72-7400D9EBB93D}">
+  <dimension ref="C1:F6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <f>C2</f>
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <f>C2*LOG(C2,2)</f>
+        <v>33.219280948873624</v>
+      </c>
+      <c r="F2">
+        <f>C2*C2</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C3">
+        <v>20</v>
+      </c>
+      <c r="D3">
+        <f t="shared" ref="D3:D6" si="0">C3</f>
+        <v>20</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E6" si="1">C3*LOG(C3,2)</f>
+        <v>86.438561897747249</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F6" si="2">C3*C3</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C4">
+        <v>30</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>147.20671786825557</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="2"/>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="5" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C5">
+        <v>40</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>212.8771237954945</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="2"/>
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="6" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <v>50</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>282.1928094887362</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="2"/>
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>